<commit_message>
Pushing changes related to the directory and file names and other code changes
</commit_message>
<xml_diff>
--- a/input/Inputfile_1.xlsx
+++ b/input/Inputfile_1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bvams\PycharmProjects\salesforce-files-downloader-tool\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bvams\PycharmProjects\salesforce-files-downloader-tool\robot\salesforce-files-downloader-tool\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35E5B97D-79EB-4819-8AAB-0F7AF2846382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66674210-8475-4940-A116-B904E49384AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,9 +25,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>ContentDocumentID</t>
+  </si>
+  <si>
+    <t>069fj000005fz33AAA</t>
+  </si>
+  <si>
+    <t>069fj000005fyrlAAA</t>
+  </si>
+  <si>
+    <t>069fj000005eLu5AAE</t>
   </si>
 </sst>
 </file>
@@ -394,16 +403,27 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2"/>
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2"/>
+      <c r="A3" s="2" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
+      <c r="A4" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" display="https://workbench.developerforce.com/retrieve.php?id=069fj000005fyrlAAA" xr:uid="{5008AF51-B73C-487E-8DB5-FA6F0385E948}"/>
+    <hyperlink ref="A3" r:id="rId2" display="https://workbench.developerforce.com/retrieve.php?id=069fj000005eLu5AAE" xr:uid="{898BD477-ABCB-4C32-9402-769B563FD31F}"/>
+    <hyperlink ref="A4" r:id="rId3" display="https://workbench.developerforce.com/retrieve.php?id=069fj000005fz33AAA" xr:uid="{5AF0CB3B-C090-463B-8C66-E78CD47E4340}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated Suite Teardown to remove temp files in directory
</commit_message>
<xml_diff>
--- a/input/Inputfile_1.xlsx
+++ b/input/Inputfile_1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bvams\PycharmProjects\salesforce-files-downloader-tool\robot\salesforce-files-downloader-tool\Input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bvams\PycharmProjects\salesforce-files-downloader-tool\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66674210-8475-4940-A116-B904E49384AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE5B03A8-35F8-43D1-BA23-E2864A0EC22E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,18 +25,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
   <si>
     <t>ContentDocumentID</t>
-  </si>
-  <si>
-    <t>069fj000005fz33AAA</t>
-  </si>
-  <si>
-    <t>069fj000005fyrlAAA</t>
-  </si>
-  <si>
-    <t>069fj000005eLu5AAE</t>
   </si>
 </sst>
 </file>
@@ -403,27 +394,16 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>2</v>
-      </c>
+      <c r="A2" s="2"/>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>3</v>
-      </c>
+      <c r="A3" s="2"/>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A4" s="2"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="https://workbench.developerforce.com/retrieve.php?id=069fj000005fyrlAAA" xr:uid="{5008AF51-B73C-487E-8DB5-FA6F0385E948}"/>
-    <hyperlink ref="A3" r:id="rId2" display="https://workbench.developerforce.com/retrieve.php?id=069fj000005eLu5AAE" xr:uid="{898BD477-ABCB-4C32-9402-769B563FD31F}"/>
-    <hyperlink ref="A4" r:id="rId3" display="https://workbench.developerforce.com/retrieve.php?id=069fj000005fz33AAA" xr:uid="{5AF0CB3B-C090-463B-8C66-E78CD47E4340}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: improve ContentDocument validation and download error handling
</commit_message>
<xml_diff>
--- a/input/Inputfile_1.xlsx
+++ b/input/Inputfile_1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bvams\PycharmProjects\salesforce-files-downloader-tool\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE5B03A8-35F8-43D1-BA23-E2864A0EC22E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23BF5199-8C64-4BB8-A91E-5582D39B400C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>